<commit_message>
Updated revised manuscript files
</commit_message>
<xml_diff>
--- a/manuscript/revision/Dataset S4.xlsx
+++ b/manuscript/revision/Dataset S4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyleewart/Documents/PostDoc/HGT_pipeline/manuscript/revision/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kewart/Downloads/revision_now/submitted/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2680C948-0D98-CB40-BB85-6C623651EC62}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81BEDD39-8256-0C4C-9238-6C3952D43787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1160" windowWidth="26900" windowHeight="16840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -164,7 +164,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -308,7 +308,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -488,8 +488,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -604,6 +610,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -649,17 +670,18 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1017,7 +1039,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="31" customWidth="1"/>
     <col min="3" max="3" width="17.1640625" bestFit="1" customWidth="1"/>
@@ -1026,453 +1048,453 @@
     <col min="7" max="7" width="39.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22" customHeight="1">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2" t="s">
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" ht="34" customHeight="1">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="3" t="s">
+      <c r="G1" s="3"/>
+    </row>
+    <row r="2" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="5" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>1037.213352</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="1">
         <v>0.50346146700000005</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="1">
         <v>14</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="1">
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <v>217.07788410000001</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="1">
         <v>0.23220464599999999</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="1">
         <v>17</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="1">
         <v>88.235294117647101</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="1">
         <v>279.945021</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="1">
         <v>0.13164256499999999</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="1">
         <v>23</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="1">
         <v>91.304347826086996</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="1">
         <v>5750.267992</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="1">
         <v>6.9512994999999994E-2</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="1">
         <v>299</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="1">
         <v>90.635451505016704</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="1">
         <v>1946.378031</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="1">
         <v>2.3480351E-2</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="1">
         <v>584</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="1">
         <v>90.753424657534296</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="1">
         <v>1471.5866329999999</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="1">
         <v>2.9350658000000002E-2</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="1">
         <v>339</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="1">
         <v>87.610619469026503</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="1">
         <v>0.414289142</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="1">
         <v>0.87571242900000001</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="1">
         <v>0.18580660700000001</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="1">
         <v>17</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
-      <c r="A10" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="1">
         <v>2664.8385199999998</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="1">
         <v>0.277923904</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="1">
         <v>20</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="1">
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
-      <c r="A11" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="1">
         <v>759.22010509999996</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="1">
         <v>4.3885286000000003E-2</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="1">
         <v>182</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="1">
         <v>87.912087912087898</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
-      <c r="A12" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="1">
         <v>1900.9342329999999</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="1">
         <v>3.9124924999999998E-2</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="1">
         <v>361</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="1">
         <v>94.459833795013907</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
-      <c r="A13" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="1">
         <v>2462.4018489999999</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="1">
         <v>3.1968934999999997E-2</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="1">
         <v>474</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="1">
         <v>91.561181434599106</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
-      <c r="A14" t="s">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="1">
         <v>2152.9058620000001</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="1">
         <v>2.6843694000000001E-2</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="1">
         <v>541</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="1">
         <v>90.757855822550795</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="1">
         <v>2467.470937</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="1">
         <v>3.0645723E-2</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="1">
         <v>465</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="1">
         <v>89.892473118279597</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="1">
         <v>2754.3200959999999</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="1">
         <v>3.290498E-2</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="1">
         <v>464</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="1">
         <v>89.870689655172399</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="1">
         <v>25.824339949999999</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="1">
         <v>0.25417458300000001</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="1">
         <v>6.3842079999999995E-2</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="1">
         <v>23</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="1">
         <v>91.304347826086996</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
-      <c r="A18" t="s">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="1">
         <v>0.111326732</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="1">
         <v>1</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="1">
         <v>0.16682830400000001</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="1">
         <v>0</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
-      <c r="A19" t="s">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="1">
         <v>57.513207719999997</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="1">
         <v>4.6895310000000003E-2</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="1">
         <v>0.12782401800000001</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="1">
         <v>5</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="1">
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
-      <c r="A20" t="s">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="1">
         <v>602.93070230000001</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>1E-4</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="1">
         <v>9.1191154999999996E-2</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="1">
         <v>79</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="1">
         <v>93.670886075949397</v>
       </c>
     </row>

</xml_diff>